<commit_message>
Update housekeeping staff roster: Ms. Arputhamani (MBA Hostel), Mr. R. Sakthivelan (Sports Hostel), Ms. Revathi (Toulouse Arena)
</commit_message>
<xml_diff>
--- a/Hostel_Housekeeping_Attendance_and_Payroll.xlsx
+++ b/Hostel_Housekeeping_Attendance_and_Payroll.xlsx
@@ -71,7 +71,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001F497D"/>
-      <sz val="14"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="6">
@@ -601,19 +601,19 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SUNSHINE HOSTEL &amp; RESIDENCY</t>
+          <t>HOSTEL &amp; FACILITY HOUSEKEEPING MANAGEMENT</t>
         </is>
       </c>
     </row>
@@ -638,14 +638,14 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>Assigned Location / Hostel</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
           <t>Designation</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Contact No.</t>
-        </is>
-      </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Monthly Base Wage (₹)</t>
@@ -658,7 +658,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Weekly Off Day</t>
+          <t>Weekly Off</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -680,21 +680,21 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Ramesh Kumar</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Head Housekeeper / Floors</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>+91 98765 43210</t>
+          <t>Ms. Arputhamani</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>MBA Hostel</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Housekeeper / MBA Hostel</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>12000</v>
+        <v>11000</v>
       </c>
       <c r="F5" s="7">
         <f>E5/31</f>
@@ -707,12 +707,12 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Bank Transfer / UPI</t>
+          <t>Bank / Cash</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>A/C: 987654321012, IFSC: SBIN0001234</t>
+          <t>MBA Hostel Desk</t>
         </is>
       </c>
     </row>
@@ -724,21 +724,21 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Sunita Devi</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Housekeeper / Rooms &amp; Corridors</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>+91 98765 43211</t>
+          <t>Mr. R. Sakthivelan</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Sports Hostel</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Housekeeper / Sports Hostel</t>
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>10500</v>
+        <v>11000</v>
       </c>
       <c r="F6" s="7">
         <f>E6/31</f>
@@ -751,12 +751,12 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Cash / Hand</t>
+          <t>Bank / Cash</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>Cash Payment Register</t>
+          <t>Sports Hostel Desk</t>
         </is>
       </c>
     </row>
@@ -768,21 +768,21 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Anil Sharma</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Housekeeper / Washrooms &amp; Common Areas</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>+91 98765 43212</t>
+          <t>Ms. Revathi</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Toulouse Arena</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Housekeeper / Toulouse Arena</t>
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>10500</v>
+        <v>11000</v>
       </c>
       <c r="F7" s="7">
         <f>E7/31</f>
@@ -795,12 +795,12 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>UPI</t>
+          <t>Bank / Cash</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>UPI ID: anilsharma@okaxis</t>
+          <t>Toulouse Arena Desk</t>
         </is>
       </c>
     </row>
@@ -816,14 +816,14 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>1. Printable_Sign_Sheet: Print this sheet at the start of the month and pin to the housekeeping notice board.</t>
+          <t>1. Printable_Sign_Sheet: Print at the start of the month and display at respective hostel/arena housekeeping desks.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>2. Attendance_Log: Record daily attendance (P = Present, A = Absent, HD = Half Day, WO = Weekly Off, PL = Paid Leave).</t>
+          <t>2. Attendance_Log: Daily attendance (P = Present, HD = Half Day, WO = Weekly Off, PL = Paid Leave, A = Absent).</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>4. Salary_Slips: Formatted payment receipts ready to print and sign upon wage disbursement.</t>
+          <t>4. Ready for wage disbursement with signature acknowledgement.</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SUNSHINE HOSTEL &amp; RESIDENCY</t>
+          <t>HOSTEL &amp; FACILITY HOUSEKEEPING MANAGEMENT</t>
         </is>
       </c>
     </row>
@@ -895,17 +895,17 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Ramesh Kumar (HK-01)</t>
+          <t>Ms. Arputhamani [MBA Hostel]</t>
         </is>
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>Sunita Devi (HK-02)</t>
+          <t>Mr. R. Sakthivelan [Sports Hostel]</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Anil Sharma (HK-03)</t>
+          <t>Ms. Revathi [Toulouse Arena]</t>
         </is>
       </c>
     </row>
@@ -1720,12 +1720,12 @@
     <row r="40">
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>Housekeeping Supervisor Signature: _______________________</t>
+          <t>Housekeeping Supervisor: _______________________</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
-          <t>Hostel Warden / Manager Signature: _______________________</t>
+          <t>Hostel Warden / Manager: _______________________</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="4.5" customWidth="1" min="4" max="4"/>
     <col width="4.5" customWidth="1" min="5" max="5"/>
     <col width="4.5" customWidth="1" min="6" max="6"/>
@@ -1799,7 +1799,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SUNSHINE HOSTEL &amp; RESIDENCY</t>
+          <t>HOSTEL &amp; FACILITY HOUSEKEEPING MANAGEMENT</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1855,7 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
@@ -2222,12 +2222,12 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Ramesh Kumar</t>
+          <t>Ms. Arputhamani</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Head Housekeeper / Floors</t>
+          <t>MBA Hostel</t>
         </is>
       </c>
       <c r="D8" s="22" t="inlineStr">
@@ -2418,12 +2418,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Sunita Devi</t>
+          <t>Mr. R. Sakthivelan</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Housekeeper / Rooms &amp; Corridors</t>
+          <t>Sports Hostel</t>
         </is>
       </c>
       <c r="D9" s="22" t="inlineStr">
@@ -2614,12 +2614,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Anil Sharma</t>
+          <t>Ms. Revathi</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Housekeeper / Washrooms &amp; Common Areas</t>
+          <t>Toulouse Arena</t>
         </is>
       </c>
       <c r="D10" s="22" t="inlineStr">
@@ -2818,14 +2818,14 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="49" customWidth="1" min="6" max="6"/>
     <col width="25" customWidth="1" min="7" max="7"/>
     <col width="36" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="53" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
@@ -2834,7 +2834,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SUNSHINE HOSTEL &amp; RESIDENCY</t>
+          <t>HOSTEL &amp; FACILITY HOUSEKEEPING MANAGEMENT</t>
         </is>
       </c>
     </row>
@@ -2859,7 +2859,7 @@
       </c>
       <c r="C4" s="26" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="D4" s="26" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>Approved By (Warden/Manager): ___________________</t>
+          <t>Sanctioned By (Warden/Manager): ___________________</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove Prepared By, Verified By, and Sanctioned By bottom signatures from remuneration sheet
</commit_message>
<xml_diff>
--- a/Hostel_Housekeeping_Attendance_and_Payroll.xlsx
+++ b/Hostel_Housekeeping_Attendance_and_Payroll.xlsx
@@ -2813,7 +2813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2821,11 +2821,11 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="49" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
     <col width="25" customWidth="1" min="7" max="7"/>
     <col width="36" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
@@ -3094,25 +3094,6 @@
       <c r="L8" s="33" t="n"/>
       <c r="M8" s="33" t="n"/>
     </row>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11">
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Prepared By: ___________________</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Verified By (Supervisor): ___________________</t>
-        </is>
-      </c>
-      <c r="J11" s="8" t="inlineStr">
-        <is>
-          <t>Sanctioned By (Warden/Manager): ___________________</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A8:C8"/>

</xml_diff>

<commit_message>
Add Legal/A4 paper size selection, enhance print clarity with crisp borders, remove bottom signatures from sign-in sheet
</commit_message>
<xml_diff>
--- a/Hostel_Housekeeping_Attendance_and_Payroll.xlsx
+++ b/Hostel_Housekeeping_Attendance_and_Payroll.xlsx
@@ -852,7 +852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1716,18 +1716,6 @@
       </c>
       <c r="J37" s="17" t="n"/>
       <c r="K37" s="17" t="n"/>
-    </row>
-    <row r="40">
-      <c r="B40" s="8" t="inlineStr">
-        <is>
-          <t>Housekeeping Supervisor: _______________________</t>
-        </is>
-      </c>
-      <c r="G40" s="8" t="inlineStr">
-        <is>
-          <t>Hostel Warden / Manager: _______________________</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
Leave Total Present Days blank on printable sheet for manual pen signing
</commit_message>
<xml_diff>
--- a/Hostel_Housekeeping_Attendance_and_Payroll.xlsx
+++ b/Hostel_Housekeeping_Attendance_and_Payroll.xlsx
@@ -1698,21 +1698,24 @@
         </is>
       </c>
       <c r="B37" s="17" t="n"/>
-      <c r="C37" s="16">
-        <f>COUNTIF(E6:E36, "P") + COUNTIF(E6:E36, "HD")*0.5</f>
-        <v/>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>________________ Days</t>
+        </is>
       </c>
       <c r="D37" s="17" t="n"/>
       <c r="E37" s="17" t="n"/>
-      <c r="F37" s="16">
-        <f>COUNTIF(H6:H36, "P") + COUNTIF(H6:H36, "HD")*0.5</f>
-        <v/>
+      <c r="F37" s="16" t="inlineStr">
+        <is>
+          <t>________________ Days</t>
+        </is>
       </c>
       <c r="G37" s="17" t="n"/>
       <c r="H37" s="17" t="n"/>
-      <c r="I37" s="16">
-        <f>COUNTIF(K6:K36, "P") + COUNTIF(K6:K36, "HD")*0.5</f>
-        <v/>
+      <c r="I37" s="16" t="inlineStr">
+        <is>
+          <t>________________ Days</t>
+        </is>
       </c>
       <c r="J37" s="17" t="n"/>
       <c r="K37" s="17" t="n"/>

</xml_diff>